<commit_message>
Add category dropdown to product import template
</commit_message>
<xml_diff>
--- a/client/public/product_import_template.xlsx
+++ b/client/public/product_import_template.xlsx
@@ -131,7 +131,7 @@
     <t>90092LR</t>
   </si>
   <si>
-    <t>RING</t>
+    <t>Rings</t>
   </si>
   <si>
     <t>18KT</t>
@@ -1921,6 +1921,11 @@
       <c r="M15" s="1"/>
     </row>
   </sheetData>
+  <dataValidations count="1">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid category" error="Pick a category from the list." promptTitle="Category" prompt="Choose from the dropdown." sqref="E2:E1000">
+      <formula1>"Bangles,Bracelets,Earrings,Necklaces,Pendants,Rings"</formula1>
+    </dataValidation>
+  </dataValidations>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <headerFooter/>
 </worksheet>

</xml_diff>

<commit_message>
add type category and sub category import, export - backend and frontend and migration
</commit_message>
<xml_diff>
--- a/client/public/product_import_template.xlsx
+++ b/client/public/product_import_template.xlsx
@@ -27,7 +27,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="111" uniqueCount="72">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="123" uniqueCount="79">
   <si>
     <t>name</t>
   </si>
@@ -44,6 +44,12 @@
     <t>category</t>
   </si>
   <si>
+    <t>type category</t>
+  </si>
+  <si>
+    <t>sub category</t>
+  </si>
+  <si>
     <t>base_price</t>
   </si>
   <si>
@@ -131,7 +137,13 @@
     <t>90092LR</t>
   </si>
   <si>
-    <t>Rings</t>
+    <t>NECKLACE SET NECKLACE</t>
+  </si>
+  <si>
+    <t>DIAMOND</t>
+  </si>
+  <si>
+    <t>LADIES</t>
   </si>
   <si>
     <t>18KT</t>
@@ -177,6 +189,9 @@
     <t>90093LR</t>
   </si>
   <si>
+    <t>RING</t>
+  </si>
+  <si>
     <t>01250496.png</t>
   </si>
   <si>
@@ -213,6 +228,9 @@
     <t>30821LR</t>
   </si>
   <si>
+    <t>JHUMKA</t>
+  </si>
+  <si>
     <t>SOLITAIRE</t>
   </si>
   <si>
@@ -232,6 +250,9 @@
   </si>
   <si>
     <t>30494DLR</t>
+  </si>
+  <si>
+    <t>COCKTAIL</t>
   </si>
   <si>
     <t>LAB GROWN</t>
@@ -1210,47 +1231,48 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
   <sheetPr/>
-  <dimension ref="A1:AH15"/>
+  <dimension ref="A1:AJ15"/>
   <sheetFormatPr defaultColWidth="9" defaultRowHeight="14.4"/>
   <cols>
     <col min="1" max="1" width="6" customWidth="1"/>
     <col min="2" max="2" width="9" style="1" customWidth="1"/>
     <col min="3" max="3" width="9.13888888888889" customWidth="1"/>
     <col min="4" max="4" width="11" customWidth="1"/>
-    <col min="5" max="5" width="8.57407407407407" customWidth="1"/>
-    <col min="6" max="6" width="10.5740740740741" customWidth="1"/>
-    <col min="7" max="7" width="11.1388888888889" customWidth="1"/>
-    <col min="8" max="8" width="11.4259259259259" customWidth="1"/>
-    <col min="9" max="9" width="12.1388888888889" customWidth="1"/>
-    <col min="10" max="10" width="10.5740740740741" customWidth="1"/>
-    <col min="11" max="11" width="14" customWidth="1"/>
-    <col min="12" max="12" width="15.287037037037" customWidth="1"/>
-    <col min="13" max="13" width="13.4259259259259" customWidth="1"/>
-    <col min="14" max="14" width="14.4259259259259" customWidth="1"/>
-    <col min="15" max="15" width="15.4259259259259" customWidth="1"/>
-    <col min="16" max="16" width="20.8518518518519" customWidth="1"/>
-    <col min="17" max="17" width="3.85185185185185" customWidth="1"/>
-    <col min="18" max="18" width="5.28703703703704" customWidth="1"/>
-    <col min="19" max="19" width="12.1388888888889" customWidth="1"/>
-    <col min="20" max="20" width="8.71296296296296" customWidth="1"/>
-    <col min="21" max="21" width="10.5740740740741" customWidth="1"/>
-    <col min="22" max="22" width="11.1388888888889" customWidth="1"/>
-    <col min="23" max="23" width="17.712962962963" customWidth="1"/>
-    <col min="24" max="24" width="18.8518518518519" customWidth="1"/>
-    <col min="25" max="25" width="3.85185185185185" customWidth="1"/>
-    <col min="26" max="26" width="5.28703703703704" customWidth="1"/>
-    <col min="27" max="27" width="10.712962962963" customWidth="1"/>
-    <col min="28" max="28" width="15.1388888888889" customWidth="1"/>
-    <col min="29" max="29" width="14.287037037037" customWidth="1"/>
-    <col min="30" max="30" width="14.5740740740741" customWidth="1"/>
-    <col min="31" max="31" width="7.28703703703704" customWidth="1"/>
-    <col min="32" max="32" width="13.287037037037" customWidth="1"/>
-    <col min="33" max="33" width="13.8518518518519" customWidth="1"/>
-    <col min="34" max="34" width="12.8518518518519" customWidth="1"/>
-    <col min="35" max="16384" width="9.13888888888889" style="2"/>
+    <col min="5" max="5" width="22.8888888888889" customWidth="1"/>
+    <col min="6" max="7" width="18.3333333333333" customWidth="1"/>
+    <col min="8" max="8" width="10.5740740740741" customWidth="1"/>
+    <col min="9" max="9" width="11.1388888888889" customWidth="1"/>
+    <col min="10" max="10" width="11.4259259259259" customWidth="1"/>
+    <col min="11" max="11" width="12.1388888888889" customWidth="1"/>
+    <col min="12" max="12" width="10.5740740740741" customWidth="1"/>
+    <col min="13" max="13" width="14" customWidth="1"/>
+    <col min="14" max="14" width="15.287037037037" customWidth="1"/>
+    <col min="15" max="15" width="13.4259259259259" customWidth="1"/>
+    <col min="16" max="16" width="14.4259259259259" customWidth="1"/>
+    <col min="17" max="17" width="15.4259259259259" customWidth="1"/>
+    <col min="18" max="18" width="20.8518518518519" customWidth="1"/>
+    <col min="19" max="19" width="3.85185185185185" customWidth="1"/>
+    <col min="20" max="20" width="5.28703703703704" customWidth="1"/>
+    <col min="21" max="21" width="12.1388888888889" customWidth="1"/>
+    <col min="22" max="22" width="8.71296296296296" customWidth="1"/>
+    <col min="23" max="23" width="10.5740740740741" customWidth="1"/>
+    <col min="24" max="24" width="11.1388888888889" customWidth="1"/>
+    <col min="25" max="25" width="17.712962962963" customWidth="1"/>
+    <col min="26" max="26" width="18.8518518518519" customWidth="1"/>
+    <col min="27" max="27" width="3.85185185185185" customWidth="1"/>
+    <col min="28" max="28" width="5.28703703703704" customWidth="1"/>
+    <col min="29" max="29" width="10.712962962963" customWidth="1"/>
+    <col min="30" max="30" width="15.1388888888889" customWidth="1"/>
+    <col min="31" max="31" width="14.287037037037" customWidth="1"/>
+    <col min="32" max="32" width="14.5740740740741" customWidth="1"/>
+    <col min="33" max="33" width="7.28703703703704" customWidth="1"/>
+    <col min="34" max="34" width="13.287037037037" customWidth="1"/>
+    <col min="35" max="35" width="13.8518518518519" customWidth="1"/>
+    <col min="36" max="36" width="12.8518518518519" customWidth="1"/>
+    <col min="37" max="16384" width="9.13888888888889" style="2"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:34">
+    <row r="1" spans="1:36">
       <c r="A1" s="3" t="s">
         <v>0</v>
       </c>
@@ -1275,37 +1297,37 @@
       <c r="H1" s="3" t="s">
         <v>7</v>
       </c>
-      <c r="I1" s="5" t="s">
+      <c r="I1" s="3" t="s">
         <v>8</v>
       </c>
-      <c r="J1" s="5" t="s">
+      <c r="J1" s="3" t="s">
         <v>9</v>
       </c>
-      <c r="K1" s="3" t="s">
+      <c r="K1" s="5" t="s">
         <v>10</v>
       </c>
-      <c r="L1" s="3" t="s">
+      <c r="L1" s="5" t="s">
         <v>11</v>
       </c>
-      <c r="M1" s="5" t="s">
+      <c r="M1" s="3" t="s">
         <v>12</v>
       </c>
       <c r="N1" s="3" t="s">
         <v>13</v>
       </c>
-      <c r="O1" s="3" t="s">
+      <c r="O1" s="5" t="s">
         <v>14</v>
       </c>
       <c r="P1" s="3" t="s">
         <v>15</v>
       </c>
-      <c r="Q1" s="5" t="s">
+      <c r="Q1" s="3" t="s">
         <v>16</v>
       </c>
       <c r="R1" s="3" t="s">
         <v>17</v>
       </c>
-      <c r="S1" s="3" t="s">
+      <c r="S1" s="5" t="s">
         <v>18</v>
       </c>
       <c r="T1" s="3" t="s">
@@ -1323,17 +1345,17 @@
       <c r="X1" s="3" t="s">
         <v>23</v>
       </c>
-      <c r="Y1" s="5" t="s">
-        <v>16</v>
-      </c>
-      <c r="Z1" s="5" t="s">
-        <v>17</v>
-      </c>
-      <c r="AA1" s="3" t="s">
+      <c r="Y1" s="3" t="s">
         <v>24</v>
       </c>
-      <c r="AB1" s="3" t="s">
+      <c r="Z1" s="3" t="s">
         <v>25</v>
+      </c>
+      <c r="AA1" s="5" t="s">
+        <v>18</v>
+      </c>
+      <c r="AB1" s="5" t="s">
+        <v>19</v>
       </c>
       <c r="AC1" s="3" t="s">
         <v>26</v>
@@ -1353,86 +1375,98 @@
       <c r="AH1" s="3" t="s">
         <v>31</v>
       </c>
+      <c r="AI1" s="3" t="s">
+        <v>32</v>
+      </c>
+      <c r="AJ1" s="3" t="s">
+        <v>33</v>
+      </c>
     </row>
-    <row r="2" ht="28.8" spans="1:34">
+    <row r="2" ht="28.8" spans="1:36">
       <c r="A2" s="3"/>
       <c r="B2" s="4" t="s">
-        <v>32</v>
+        <v>34</v>
       </c>
       <c r="C2" s="3" t="s">
-        <v>33</v>
+        <v>35</v>
       </c>
       <c r="D2" s="3"/>
       <c r="E2" s="3" t="s">
-        <v>34</v>
-      </c>
-      <c r="F2" s="3"/>
+        <v>36</v>
+      </c>
+      <c r="F2" s="3" t="s">
+        <v>37</v>
+      </c>
       <c r="G2" s="3" t="s">
-        <v>35</v>
-      </c>
-      <c r="H2" s="3" t="s">
-        <v>36</v>
-      </c>
-      <c r="I2" s="6">
+        <v>38</v>
+      </c>
+      <c r="H2" s="3"/>
+      <c r="I2" s="3" t="s">
+        <v>39</v>
+      </c>
+      <c r="J2" s="3" t="s">
+        <v>40</v>
+      </c>
+      <c r="K2" s="6">
         <v>1.63</v>
       </c>
-      <c r="J2" s="6">
+      <c r="L2" s="6">
         <v>1.594</v>
       </c>
-      <c r="K2" s="3" t="s">
-        <v>37</v>
-      </c>
-      <c r="L2" s="3" t="s">
-        <v>38</v>
-      </c>
-      <c r="M2" s="4" t="s">
-        <v>39</v>
+      <c r="M2" s="3" t="s">
+        <v>41</v>
       </c>
       <c r="N2" s="3" t="s">
-        <v>40</v>
-      </c>
-      <c r="O2" s="3" t="s">
-        <v>41</v>
+        <v>42</v>
+      </c>
+      <c r="O2" s="4" t="s">
+        <v>43</v>
       </c>
       <c r="P2" s="3" t="s">
-        <v>42</v>
-      </c>
-      <c r="Q2" s="3">
+        <v>44</v>
+      </c>
+      <c r="Q2" s="3" t="s">
+        <v>45</v>
+      </c>
+      <c r="R2" s="3" t="s">
+        <v>46</v>
+      </c>
+      <c r="S2" s="3">
         <v>1</v>
       </c>
-      <c r="R2" s="7">
+      <c r="T2" s="7">
         <v>0.03</v>
       </c>
-      <c r="S2" s="3"/>
-      <c r="T2" s="3"/>
       <c r="U2" s="3"/>
       <c r="V2" s="3"/>
       <c r="W2" s="3"/>
       <c r="X2" s="3"/>
       <c r="Y2" s="3"/>
       <c r="Z2" s="3"/>
-      <c r="AA2" s="3" t="s">
-        <v>43</v>
-      </c>
-      <c r="AB2" s="3">
+      <c r="AA2" s="3"/>
+      <c r="AB2" s="3"/>
+      <c r="AC2" s="3" t="s">
+        <v>47</v>
+      </c>
+      <c r="AD2" s="3">
         <v>7</v>
       </c>
-      <c r="AC2" s="3">
+      <c r="AE2" s="3">
         <v>1</v>
       </c>
-      <c r="AD2" s="3">
+      <c r="AF2" s="3">
         <v>100</v>
       </c>
-      <c r="AE2" s="3" t="b">
+      <c r="AG2" s="3" t="b">
         <v>1</v>
       </c>
-      <c r="AF2" s="3"/>
-      <c r="AG2" s="3"/>
-      <c r="AH2" s="8" t="s">
-        <v>44</v>
+      <c r="AH2" s="3"/>
+      <c r="AI2" s="3"/>
+      <c r="AJ2" s="8" t="s">
+        <v>48</v>
       </c>
     </row>
-    <row r="3" spans="1:34">
+    <row r="3" spans="1:36">
       <c r="A3" s="3"/>
       <c r="B3" s="4"/>
       <c r="C3" s="3"/>
@@ -1441,32 +1475,32 @@
       <c r="F3" s="3"/>
       <c r="G3" s="3"/>
       <c r="H3" s="3"/>
-      <c r="I3" s="6"/>
-      <c r="J3" s="6"/>
-      <c r="K3" s="3" t="s">
-        <v>37</v>
-      </c>
-      <c r="L3" s="3" t="s">
+      <c r="I3" s="3"/>
+      <c r="J3" s="3"/>
+      <c r="K3" s="6"/>
+      <c r="L3" s="6"/>
+      <c r="M3" s="3" t="s">
+        <v>41</v>
+      </c>
+      <c r="N3" s="3" t="s">
+        <v>49</v>
+      </c>
+      <c r="O3" s="4" t="s">
+        <v>50</v>
+      </c>
+      <c r="P3" s="3" t="s">
+        <v>44</v>
+      </c>
+      <c r="Q3" s="3" t="s">
         <v>45</v>
       </c>
-      <c r="M3" s="4" t="s">
-        <v>46</v>
-      </c>
-      <c r="N3" s="3" t="s">
-        <v>40</v>
-      </c>
-      <c r="O3" s="3" t="s">
-        <v>41</v>
-      </c>
-      <c r="P3" s="3"/>
-      <c r="Q3" s="3">
+      <c r="R3" s="3"/>
+      <c r="S3" s="3">
         <v>27</v>
       </c>
-      <c r="R3" s="7">
+      <c r="T3" s="7">
         <v>0.15</v>
       </c>
-      <c r="S3" s="3"/>
-      <c r="T3" s="3"/>
       <c r="U3" s="3"/>
       <c r="V3" s="3"/>
       <c r="W3" s="3"/>
@@ -1477,92 +1511,100 @@
       <c r="AB3" s="3"/>
       <c r="AC3" s="3"/>
       <c r="AD3" s="3"/>
-      <c r="AE3" s="3" t="b">
+      <c r="AE3" s="3"/>
+      <c r="AF3" s="3"/>
+      <c r="AG3" s="3" t="b">
         <v>1</v>
       </c>
-      <c r="AF3" s="3"/>
-      <c r="AG3" s="3"/>
       <c r="AH3" s="3"/>
+      <c r="AI3" s="3"/>
+      <c r="AJ3" s="3"/>
     </row>
-    <row r="4" spans="1:34">
+    <row r="4" spans="1:36">
       <c r="A4" s="3"/>
       <c r="B4" s="4" t="s">
-        <v>47</v>
+        <v>51</v>
       </c>
       <c r="C4" s="3" t="s">
-        <v>48</v>
+        <v>52</v>
       </c>
       <c r="D4" s="3"/>
       <c r="E4" s="3" t="s">
-        <v>34</v>
-      </c>
-      <c r="F4" s="3"/>
+        <v>53</v>
+      </c>
+      <c r="F4" s="3" t="s">
+        <v>37</v>
+      </c>
       <c r="G4" s="3" t="s">
-        <v>35</v>
-      </c>
-      <c r="H4" s="3" t="s">
-        <v>36</v>
-      </c>
-      <c r="I4" s="6">
+        <v>38</v>
+      </c>
+      <c r="H4" s="3"/>
+      <c r="I4" s="3" t="s">
+        <v>39</v>
+      </c>
+      <c r="J4" s="3" t="s">
+        <v>40</v>
+      </c>
+      <c r="K4" s="6">
         <v>1.42</v>
       </c>
-      <c r="J4" s="6">
+      <c r="L4" s="6">
         <v>1.382</v>
       </c>
-      <c r="K4" s="3" t="s">
-        <v>37</v>
-      </c>
-      <c r="L4" s="3" t="s">
-        <v>38</v>
-      </c>
-      <c r="M4" s="4" t="s">
-        <v>39</v>
+      <c r="M4" s="3" t="s">
+        <v>41</v>
       </c>
       <c r="N4" s="3" t="s">
-        <v>40</v>
-      </c>
-      <c r="O4" s="3" t="s">
-        <v>41</v>
+        <v>42</v>
+      </c>
+      <c r="O4" s="4" t="s">
+        <v>43</v>
       </c>
       <c r="P4" s="3" t="s">
-        <v>42</v>
-      </c>
-      <c r="Q4" s="3">
+        <v>44</v>
+      </c>
+      <c r="Q4" s="3" t="s">
+        <v>45</v>
+      </c>
+      <c r="R4" s="3" t="s">
+        <v>46</v>
+      </c>
+      <c r="S4" s="3">
         <v>1</v>
       </c>
-      <c r="R4" s="7">
+      <c r="T4" s="7">
         <v>0.03</v>
       </c>
-      <c r="S4" s="3"/>
-      <c r="T4" s="3"/>
       <c r="U4" s="3"/>
       <c r="V4" s="3"/>
       <c r="W4" s="3"/>
       <c r="X4" s="3"/>
       <c r="Y4" s="3"/>
       <c r="Z4" s="3"/>
-      <c r="AA4" s="3" t="s">
-        <v>43</v>
-      </c>
-      <c r="AB4" s="3">
+      <c r="AA4" s="3"/>
+      <c r="AB4" s="3"/>
+      <c r="AC4" s="3" t="s">
+        <v>47</v>
+      </c>
+      <c r="AD4" s="3">
         <v>7</v>
       </c>
-      <c r="AC4" s="3">
+      <c r="AE4" s="3">
         <v>1</v>
       </c>
-      <c r="AD4" s="3">
+      <c r="AF4" s="3">
         <v>100</v>
       </c>
-      <c r="AE4" s="3" t="b">
+      <c r="AG4" s="3" t="b">
         <v>1</v>
       </c>
-      <c r="AF4" s="3"/>
-      <c r="AG4" s="3"/>
-      <c r="AH4" s="3" t="s">
-        <v>49</v>
+      <c r="AH4" s="3"/>
+      <c r="AI4" s="3"/>
+      <c r="AJ4" s="3" t="s">
+        <v>54</v>
       </c>
     </row>
-    <row r="5" spans="1:34">
+    <row r="5" spans="1:36">
       <c r="A5" s="3"/>
       <c r="B5" s="4"/>
       <c r="C5" s="3"/>
@@ -1571,32 +1613,32 @@
       <c r="F5" s="3"/>
       <c r="G5" s="3"/>
       <c r="H5" s="3"/>
-      <c r="I5" s="6"/>
-      <c r="J5" s="6"/>
-      <c r="K5" s="3" t="s">
-        <v>37</v>
-      </c>
-      <c r="L5" s="3" t="s">
+      <c r="I5" s="3"/>
+      <c r="J5" s="3"/>
+      <c r="K5" s="6"/>
+      <c r="L5" s="6"/>
+      <c r="M5" s="3" t="s">
+        <v>41</v>
+      </c>
+      <c r="N5" s="3" t="s">
+        <v>49</v>
+      </c>
+      <c r="O5" s="4" t="s">
+        <v>50</v>
+      </c>
+      <c r="P5" s="3" t="s">
+        <v>44</v>
+      </c>
+      <c r="Q5" s="3" t="s">
         <v>45</v>
       </c>
-      <c r="M5" s="4" t="s">
-        <v>46</v>
-      </c>
-      <c r="N5" s="3" t="s">
-        <v>40</v>
-      </c>
-      <c r="O5" s="3" t="s">
-        <v>41</v>
-      </c>
-      <c r="P5" s="3"/>
-      <c r="Q5" s="3">
+      <c r="R5" s="3"/>
+      <c r="S5" s="3">
         <v>27</v>
       </c>
-      <c r="R5" s="7">
+      <c r="T5" s="7">
         <v>0.16</v>
       </c>
-      <c r="S5" s="3"/>
-      <c r="T5" s="3"/>
       <c r="U5" s="3"/>
       <c r="V5" s="3"/>
       <c r="W5" s="3"/>
@@ -1607,90 +1649,98 @@
       <c r="AB5" s="3"/>
       <c r="AC5" s="3"/>
       <c r="AD5" s="3"/>
-      <c r="AE5" s="3" t="b">
+      <c r="AE5" s="3"/>
+      <c r="AF5" s="3"/>
+      <c r="AG5" s="3" t="b">
         <v>1</v>
       </c>
-      <c r="AF5" s="3"/>
-      <c r="AG5" s="3"/>
       <c r="AH5" s="3"/>
+      <c r="AI5" s="3"/>
+      <c r="AJ5" s="3"/>
     </row>
-    <row r="6" spans="1:34">
+    <row r="6" spans="1:36">
       <c r="A6" s="3"/>
       <c r="B6" s="4" t="s">
-        <v>50</v>
+        <v>55</v>
       </c>
       <c r="C6" s="3" t="s">
-        <v>51</v>
+        <v>56</v>
       </c>
       <c r="D6" s="3"/>
       <c r="E6" s="3" t="s">
-        <v>34</v>
-      </c>
-      <c r="F6" s="3"/>
+        <v>53</v>
+      </c>
+      <c r="F6" s="3" t="s">
+        <v>37</v>
+      </c>
       <c r="G6" s="3" t="s">
-        <v>35</v>
+        <v>38</v>
       </c>
       <c r="H6" s="3"/>
-      <c r="I6" s="6">
+      <c r="I6" s="3" t="s">
+        <v>39</v>
+      </c>
+      <c r="J6" s="3"/>
+      <c r="K6" s="6">
         <v>2.67</v>
       </c>
-      <c r="J6" s="6">
+      <c r="L6" s="6">
         <v>2.504</v>
       </c>
-      <c r="K6" s="3" t="s">
-        <v>37</v>
-      </c>
-      <c r="L6" s="3" t="s">
-        <v>52</v>
-      </c>
-      <c r="M6" s="4" t="s">
-        <v>53</v>
+      <c r="M6" s="3" t="s">
+        <v>41</v>
       </c>
       <c r="N6" s="3" t="s">
-        <v>40</v>
-      </c>
-      <c r="O6" s="3" t="s">
-        <v>41</v>
+        <v>57</v>
+      </c>
+      <c r="O6" s="4" t="s">
+        <v>58</v>
       </c>
       <c r="P6" s="3" t="s">
-        <v>42</v>
-      </c>
-      <c r="Q6" s="3">
+        <v>44</v>
+      </c>
+      <c r="Q6" s="3" t="s">
+        <v>45</v>
+      </c>
+      <c r="R6" s="3" t="s">
+        <v>46</v>
+      </c>
+      <c r="S6" s="3">
         <v>4</v>
       </c>
-      <c r="R6" s="7">
+      <c r="T6" s="7">
         <v>0.16</v>
       </c>
-      <c r="S6" s="3"/>
-      <c r="T6" s="3"/>
       <c r="U6" s="3"/>
       <c r="V6" s="3"/>
       <c r="W6" s="3"/>
       <c r="X6" s="3"/>
       <c r="Y6" s="3"/>
       <c r="Z6" s="3"/>
-      <c r="AA6" s="3" t="s">
-        <v>43</v>
-      </c>
-      <c r="AB6" s="3">
+      <c r="AA6" s="3"/>
+      <c r="AB6" s="3"/>
+      <c r="AC6" s="3" t="s">
+        <v>47</v>
+      </c>
+      <c r="AD6" s="3">
         <v>7</v>
       </c>
-      <c r="AC6" s="3">
+      <c r="AE6" s="3">
         <v>1</v>
       </c>
-      <c r="AD6" s="3">
+      <c r="AF6" s="3">
         <v>100</v>
       </c>
-      <c r="AE6" s="3" t="b">
+      <c r="AG6" s="3" t="b">
         <v>1</v>
       </c>
-      <c r="AF6" s="3"/>
-      <c r="AG6" s="3"/>
-      <c r="AH6" s="3" t="s">
-        <v>54</v>
+      <c r="AH6" s="3"/>
+      <c r="AI6" s="3"/>
+      <c r="AJ6" s="3" t="s">
+        <v>59</v>
       </c>
     </row>
-    <row r="7" spans="1:34">
+    <row r="7" spans="1:36">
       <c r="A7" s="3"/>
       <c r="B7" s="4"/>
       <c r="C7" s="3"/>
@@ -1699,231 +1749,251 @@
       <c r="F7" s="3"/>
       <c r="G7" s="3"/>
       <c r="H7" s="3"/>
-      <c r="I7" s="6" t="s">
-        <v>55</v>
-      </c>
-      <c r="J7" s="6"/>
-      <c r="K7" s="3" t="s">
-        <v>37</v>
-      </c>
-      <c r="L7" s="3" t="s">
+      <c r="I7" s="3"/>
+      <c r="J7" s="3"/>
+      <c r="K7" s="6" t="s">
+        <v>60</v>
+      </c>
+      <c r="L7" s="6"/>
+      <c r="M7" s="3" t="s">
+        <v>41</v>
+      </c>
+      <c r="N7" s="3" t="s">
+        <v>49</v>
+      </c>
+      <c r="O7" s="4" t="s">
+        <v>61</v>
+      </c>
+      <c r="P7" s="3" t="s">
+        <v>44</v>
+      </c>
+      <c r="Q7" s="3" t="s">
         <v>45</v>
       </c>
-      <c r="M7" s="4" t="s">
-        <v>56</v>
-      </c>
-      <c r="N7" s="3" t="s">
-        <v>40</v>
-      </c>
-      <c r="O7" s="3" t="s">
-        <v>41</v>
-      </c>
-      <c r="P7" s="3"/>
-      <c r="Q7" s="3">
+      <c r="R7" s="3"/>
+      <c r="S7" s="3">
         <v>8</v>
       </c>
-      <c r="R7" s="7">
+      <c r="T7" s="7">
         <v>0.12</v>
       </c>
-      <c r="S7" s="3"/>
-      <c r="T7" s="3"/>
       <c r="U7" s="3"/>
       <c r="V7" s="3"/>
-      <c r="W7" s="3" t="s">
-        <v>57</v>
-      </c>
-      <c r="X7" s="3" t="s">
-        <v>58</v>
-      </c>
-      <c r="Y7" s="3">
+      <c r="W7" s="3"/>
+      <c r="X7" s="3"/>
+      <c r="Y7" s="3" t="s">
+        <v>62</v>
+      </c>
+      <c r="Z7" s="3" t="s">
+        <v>63</v>
+      </c>
+      <c r="AA7" s="3">
         <v>1</v>
       </c>
-      <c r="Z7" s="7">
+      <c r="AB7" s="7">
         <v>0.55</v>
       </c>
-      <c r="AA7" s="3"/>
-      <c r="AB7" s="3"/>
       <c r="AC7" s="3"/>
       <c r="AD7" s="3"/>
-      <c r="AE7" s="3" t="b">
+      <c r="AE7" s="3"/>
+      <c r="AF7" s="3"/>
+      <c r="AG7" s="3" t="b">
         <v>1</v>
       </c>
-      <c r="AF7" s="3"/>
-      <c r="AG7" s="3"/>
       <c r="AH7" s="3"/>
+      <c r="AI7" s="3"/>
+      <c r="AJ7" s="3"/>
     </row>
-    <row r="8" spans="1:34">
+    <row r="8" spans="1:36">
       <c r="A8" s="3"/>
       <c r="B8" s="4" t="s">
-        <v>59</v>
+        <v>64</v>
       </c>
       <c r="C8" s="3" t="s">
-        <v>60</v>
+        <v>65</v>
       </c>
       <c r="D8" s="3"/>
       <c r="E8" s="3" t="s">
-        <v>34</v>
-      </c>
-      <c r="F8" s="3"/>
+        <v>53</v>
+      </c>
+      <c r="F8" s="3" t="s">
+        <v>37</v>
+      </c>
       <c r="G8" s="3" t="s">
-        <v>35</v>
+        <v>66</v>
       </c>
       <c r="H8" s="3"/>
-      <c r="I8" s="6">
+      <c r="I8" s="3" t="s">
+        <v>39</v>
+      </c>
+      <c r="J8" s="3"/>
+      <c r="K8" s="6">
         <v>9.69</v>
       </c>
-      <c r="J8" s="6">
+      <c r="L8" s="6">
         <v>9.286</v>
       </c>
-      <c r="K8" s="3" t="s">
-        <v>37</v>
-      </c>
-      <c r="L8" s="3" t="s">
-        <v>61</v>
-      </c>
-      <c r="M8" s="4"/>
+      <c r="M8" s="3" t="s">
+        <v>41</v>
+      </c>
       <c r="N8" s="3" t="s">
-        <v>62</v>
-      </c>
-      <c r="O8" s="3" t="s">
-        <v>63</v>
-      </c>
+        <v>67</v>
+      </c>
+      <c r="O8" s="4"/>
       <c r="P8" s="3" t="s">
-        <v>64</v>
-      </c>
-      <c r="Q8" s="3">
+        <v>68</v>
+      </c>
+      <c r="Q8" s="3" t="s">
+        <v>69</v>
+      </c>
+      <c r="R8" s="3" t="s">
+        <v>70</v>
+      </c>
+      <c r="S8" s="3">
         <v>1</v>
       </c>
-      <c r="R8" s="7">
+      <c r="T8" s="7">
         <v>2.02</v>
       </c>
-      <c r="S8" s="3"/>
-      <c r="T8" s="3"/>
       <c r="U8" s="3"/>
       <c r="V8" s="3"/>
       <c r="W8" s="3"/>
       <c r="X8" s="3"/>
       <c r="Y8" s="3"/>
       <c r="Z8" s="3"/>
-      <c r="AA8" s="3" t="s">
-        <v>43</v>
-      </c>
-      <c r="AB8" s="3">
+      <c r="AA8" s="3"/>
+      <c r="AB8" s="3"/>
+      <c r="AC8" s="3" t="s">
+        <v>47</v>
+      </c>
+      <c r="AD8" s="3">
         <v>7</v>
       </c>
-      <c r="AC8" s="3">
+      <c r="AE8" s="3">
         <v>1</v>
       </c>
-      <c r="AD8" s="3">
+      <c r="AF8" s="3">
         <v>100</v>
       </c>
-      <c r="AE8" s="3" t="b">
+      <c r="AG8" s="3" t="b">
         <v>1</v>
       </c>
-      <c r="AF8" s="3"/>
-      <c r="AG8" s="3"/>
-      <c r="AH8" s="3" t="s">
-        <v>65</v>
+      <c r="AH8" s="3"/>
+      <c r="AI8" s="3"/>
+      <c r="AJ8" s="3" t="s">
+        <v>71</v>
       </c>
     </row>
-    <row r="9" spans="1:34">
+    <row r="9" spans="1:36">
       <c r="A9" s="3"/>
       <c r="B9" s="4" t="s">
-        <v>66</v>
+        <v>72</v>
       </c>
       <c r="C9" s="3" t="s">
-        <v>67</v>
+        <v>73</v>
       </c>
       <c r="D9" s="3"/>
       <c r="E9" s="3" t="s">
-        <v>34</v>
-      </c>
-      <c r="F9" s="3"/>
+        <v>53</v>
+      </c>
+      <c r="F9" s="3" t="s">
+        <v>37</v>
+      </c>
       <c r="G9" s="3" t="s">
-        <v>35</v>
+        <v>74</v>
       </c>
       <c r="H9" s="3"/>
-      <c r="I9" s="6">
+      <c r="I9" s="3" t="s">
+        <v>39</v>
+      </c>
+      <c r="J9" s="3"/>
+      <c r="K9" s="6">
         <v>6.44</v>
       </c>
-      <c r="J9" s="6">
+      <c r="L9" s="6">
         <v>6.02</v>
       </c>
-      <c r="K9" s="3" t="s">
-        <v>68</v>
-      </c>
-      <c r="L9" s="3" t="s">
-        <v>45</v>
-      </c>
-      <c r="M9" s="4"/>
-      <c r="N9" s="3"/>
-      <c r="O9" s="3"/>
+      <c r="M9" s="3" t="s">
+        <v>75</v>
+      </c>
+      <c r="N9" s="3" t="s">
+        <v>49</v>
+      </c>
+      <c r="O9" s="4"/>
       <c r="P9" s="3"/>
-      <c r="Q9" s="3">
+      <c r="Q9" s="3"/>
+      <c r="R9" s="3"/>
+      <c r="S9" s="3">
         <v>1</v>
       </c>
-      <c r="R9" s="7">
+      <c r="T9" s="7">
         <v>1.25</v>
       </c>
-      <c r="S9" s="3"/>
-      <c r="T9" s="3"/>
       <c r="U9" s="3"/>
       <c r="V9" s="3"/>
-      <c r="W9" s="3" t="s">
-        <v>69</v>
-      </c>
-      <c r="X9" s="3" t="s">
-        <v>70</v>
-      </c>
-      <c r="Y9" s="3">
+      <c r="W9" s="3"/>
+      <c r="X9" s="3"/>
+      <c r="Y9" s="3" t="s">
+        <v>76</v>
+      </c>
+      <c r="Z9" s="3" t="s">
+        <v>77</v>
+      </c>
+      <c r="AA9" s="3">
         <v>52</v>
       </c>
-      <c r="Z9" s="7">
+      <c r="AB9" s="7">
         <v>0.85</v>
       </c>
-      <c r="AA9" s="3" t="s">
-        <v>43</v>
-      </c>
-      <c r="AB9" s="3">
+      <c r="AC9" s="3" t="s">
+        <v>47</v>
+      </c>
+      <c r="AD9" s="3">
         <v>7</v>
       </c>
-      <c r="AC9" s="3">
+      <c r="AE9" s="3">
         <v>1</v>
       </c>
-      <c r="AD9" s="3">
+      <c r="AF9" s="3">
         <v>100</v>
       </c>
-      <c r="AE9" s="3" t="b">
+      <c r="AG9" s="3" t="b">
         <v>1</v>
       </c>
-      <c r="AF9" s="3"/>
-      <c r="AG9" s="3"/>
-      <c r="AH9" s="3" t="s">
-        <v>71</v>
+      <c r="AH9" s="3"/>
+      <c r="AI9" s="3"/>
+      <c r="AJ9" s="3" t="s">
+        <v>78</v>
       </c>
     </row>
-    <row r="10" spans="1:34">
-      <c r="M10" s="1"/>
+    <row r="10" spans="1:36">
+      <c r="O10" s="1"/>
     </row>
-    <row r="11" spans="1:34">
-      <c r="M11" s="1"/>
+    <row r="11" spans="1:36">
+      <c r="O11" s="1"/>
     </row>
-    <row r="12" spans="1:34">
-      <c r="M12" s="1"/>
+    <row r="12" spans="1:36">
+      <c r="O12" s="1"/>
     </row>
-    <row r="13" spans="1:34">
-      <c r="M13" s="1"/>
+    <row r="13" spans="1:36">
+      <c r="O13" s="1"/>
     </row>
-    <row r="14" spans="1:34">
-      <c r="M14" s="1"/>
+    <row r="14" spans="1:36">
+      <c r="O14" s="1"/>
     </row>
-    <row r="15" spans="1:34">
-      <c r="M15" s="1"/>
+    <row r="15" spans="1:36">
+      <c r="O15" s="1"/>
     </row>
   </sheetData>
-  <dataValidations count="1">
+  <dataValidations count="3">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="F2 F4 F6 F8 F9">
+      <formula1>" DIAMOND, GOLD, POLKI, KUNDAN"</formula1>
+    </dataValidation>
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="G2 G4 G6 G8 G9">
+      <formula1>"LADIES,3 PCS SET,BALI,COCKTAIL,GENTS,JHUMKA,KODA JODI,LADIES,SOLITAIRE,TOPS"</formula1>
+    </dataValidation>
     <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid category" error="Pick a category from the list." promptTitle="Category" prompt="Choose from the dropdown." sqref="E2:E1000">
-      <formula1>"Bangles,Bracelets,Earrings,Necklaces,Pendants,Rings"</formula1>
+      <formula1>"RING,PENDENT,EARRING,BANGLES,NAGMALA,BRACELET,PENDENT SET PENDENT,PENDENT SET EARRING,NECKLACE SET NECKLACE,NECKLACE SET EARRING,NOSEPIN,MANGALSUTRA"</formula1>
     </dataValidation>
   </dataValidations>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>